<commit_message>
docs: Update benchmark spreadsheet with full 7-model suite results on NVIDIA A100
</commit_message>
<xml_diff>
--- a/results/edge_benchmark_results.xlsx
+++ b/results/edge_benchmark_results.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -594,28 +594,28 @@
         </is>
       </c>
       <c r="F2" s="4" t="n">
-        <v>4.02</v>
+        <v>4.01</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>4.02</v>
+        <v>4.01</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>248.9</v>
+        <v>249.6</v>
       </c>
       <c r="I2" s="4" t="n">
         <v>0.35</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>3.32</v>
+        <v>3.31</v>
       </c>
       <c r="K2" s="4" t="n">
         <v>0.24</v>
       </c>
       <c r="L2" s="4" t="n">
-        <v>3.91</v>
+        <v>3.9</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>255.9</v>
+        <v>256.5</v>
       </c>
       <c r="N2" s="4" t="n">
         <v>19.88</v>
@@ -653,28 +653,28 @@
         </is>
       </c>
       <c r="F3" s="7" t="n">
-        <v>3.79</v>
+        <v>4.02</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>3.79</v>
+        <v>4.02</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>263.9</v>
+        <v>249</v>
       </c>
       <c r="I3" s="7" t="n">
         <v>0.35</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>3.42</v>
+        <v>3.43</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>0.24</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>4.01</v>
+        <v>4.02</v>
       </c>
       <c r="M3" s="7" t="n">
-        <v>249.5</v>
+        <v>248.7</v>
       </c>
       <c r="N3" s="7" t="n">
         <v>20.15</v>
@@ -688,22 +688,22 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Workstation GPU</t>
+          <t>Datacenter Cloud Server</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>NVIDIA GeForce RTX 4070 Laptop</t>
+          <t>NVIDIA A100 80GB PCIe MIG</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>NVIDIA Ada Lovelace (AD106)</t>
+          <t>NVIDIA Ampere (GA100)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Ours (Hybrid Dilated ECA v30)</t>
+          <t>Stock YOLOv8s Baseline</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -712,80 +712,375 @@
         </is>
       </c>
       <c r="F4" s="4" t="n">
-        <v>5.14</v>
+        <v>5.7</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>4.99</v>
+        <v>5.7</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>194.7</v>
+        <v>175.5</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>1.71</v>
+        <v>0.35</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>3.32</v>
+        <v>5.4</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>0.35</v>
+        <v>0.29</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>5.38</v>
+        <v>6.04</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>185.9</v>
+        <v>165.5</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>20.23</v>
+        <v>44.12</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>Verified (Local Workstation)</t>
+          <t>Verified (UiA Coder A100)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
+          <t>Datacenter Cloud Server</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>NVIDIA A100 80GB PCIe MIG</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>NVIDIA Ampere (GA100)</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Stock YOLOv10n Baseline</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>FP16</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>6.19</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>6.19</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>161.7</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="M5" s="7" t="n">
+        <v>241.3</v>
+      </c>
+      <c r="N5" s="7" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="O5" s="5" t="inlineStr">
+        <is>
+          <t>Verified (UiA Coder A100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Datacenter Cloud Server</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA A100 80GB PCIe MIG</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA Ampere (GA100)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Stock YOLOv10s Baseline</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>FP16</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>7.13</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>7.13</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>140.3</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>5.58</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>6.22</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>160.8</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>Verified (UiA Coder A100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Datacenter Cloud Server</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>NVIDIA A100 80GB PCIe MIG</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>NVIDIA Ampere (GA100)</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Stock YOLOv11n Baseline</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>FP16</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>5.34</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>5.34</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>187.2</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="K7" s="7" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <v>4.22</v>
+      </c>
+      <c r="M7" s="7" t="n">
+        <v>237.2</v>
+      </c>
+      <c r="N7" s="7" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="O7" s="5" t="inlineStr">
+        <is>
+          <t>Verified (UiA Coder A100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Datacenter Cloud Server</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA A100 80GB PCIe MIG</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA Ampere (GA100)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Stock YOLOv11s Baseline</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>FP16</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>5.86</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>5.86</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>170.7</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>5.42</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>164.9</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>Verified (UiA Coder A100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Workstation GPU</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>NVIDIA GeForce RTX 4070 Laptop</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>NVIDIA Ada Lovelace (AD106)</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Ours (Hybrid Dilated ECA v30)</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>FP16</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>5.14</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>194.7</v>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="K9" s="7" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <v>5.38</v>
+      </c>
+      <c r="M9" s="7" t="n">
+        <v>185.9</v>
+      </c>
+      <c r="N9" s="7" t="n">
+        <v>20.23</v>
+      </c>
+      <c r="O9" s="5" t="inlineStr">
+        <is>
+          <t>Verified (Local Workstation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>Host Workstation CPU</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Intel Core i7-13700H</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>x86_64 (14 Cores / 20 Threads)</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Ours (Hybrid Dilated ECA v30)</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>FP32</t>
         </is>
       </c>
-      <c r="F5" s="7" t="n">
+      <c r="F10" s="4" t="n">
         <v>63.63</v>
       </c>
-      <c r="G5" s="7" t="n">
+      <c r="G10" s="4" t="n">
         <v>63.25</v>
       </c>
-      <c r="H5" s="7" t="n">
+      <c r="H10" s="4" t="n">
         <v>15.72</v>
       </c>
-      <c r="I5" s="7" t="inlineStr"/>
-      <c r="J5" s="7" t="inlineStr"/>
-      <c r="K5" s="7" t="inlineStr"/>
-      <c r="L5" s="7" t="inlineStr"/>
-      <c r="M5" s="7" t="inlineStr"/>
-      <c r="N5" s="7" t="inlineStr"/>
-      <c r="O5" s="5" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr"/>
+      <c r="J10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="inlineStr"/>
+      <c r="L10" s="4" t="inlineStr"/>
+      <c r="M10" s="4" t="inlineStr"/>
+      <c r="N10" s="4" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr">
         <is>
           <t>Verified (Local Workstation)</t>
         </is>

</xml_diff>

<commit_message>
docs: Append AMD EPYC 9374F 32-Core CPU benchmark results for all 7 models
</commit_message>
<xml_diff>
--- a/results/edge_benchmark_results.xlsx
+++ b/results/edge_benchmark_results.xlsx
@@ -470,11 +470,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
@@ -1086,6 +1086,405 @@
         </is>
       </c>
     </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Datacenter Server CPU</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>AMD EPYC 9374F 32-Core Processor</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>x86_64 (Zen 4, 32C/64T)</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Ours (Hybrid Dilated ECA v30)</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>FP32</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>27.93</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>27.93</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="L11" s="7" t="n">
+        <v>27.93</v>
+      </c>
+      <c r="M11" s="7" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="N11" s="7" t="inlineStr"/>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>Verified (UiA Coder EPYC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Datacenter Server CPU</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>AMD EPYC 9374F 32-Core Processor</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>x86_64 (Zen 4, 32C/64T)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Stock YOLOv8n Baseline</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>FP32</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>45.38</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>45.38</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>26.12</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>28.97</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="N12" s="4" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>Verified (UiA Coder EPYC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Datacenter Server CPU</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>AMD EPYC 9374F 32-Core Processor</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>x86_64 (Zen 4, 32C/64T)</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Stock YOLOv8s Baseline</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>FP32</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>87.73</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>87.73</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="L13" s="7" t="n">
+        <v>57.85</v>
+      </c>
+      <c r="M13" s="7" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="N13" s="7" t="inlineStr"/>
+      <c r="O13" s="5" t="inlineStr">
+        <is>
+          <t>Verified (UiA Coder EPYC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Datacenter Server CPU</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>AMD EPYC 9374F 32-Core Processor</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>x86_64 (Zen 4, 32C/64T)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Stock YOLOv10n Baseline</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>FP32</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>51.35</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>51.35</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>28.05</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="N14" s="4" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>Verified (UiA Coder EPYC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Datacenter Server CPU</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>AMD EPYC 9374F 32-Core Processor</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>x86_64 (Zen 4, 32C/64T)</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Stock YOLOv10s Baseline</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>FP32</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>97.55</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>97.55</v>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="L15" s="7" t="n">
+        <v>56.86</v>
+      </c>
+      <c r="M15" s="7" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="N15" s="7" t="inlineStr"/>
+      <c r="O15" s="5" t="inlineStr">
+        <is>
+          <t>Verified (UiA Coder EPYC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Datacenter Server CPU</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>AMD EPYC 9374F 32-Core Processor</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>x86_64 (Zen 4, 32C/64T)</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Stock YOLOv11n Baseline</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>FP32</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>43.55</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>43.55</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>26.65</v>
+      </c>
+      <c r="K16" s="4" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>29.54</v>
+      </c>
+      <c r="M16" s="4" t="n">
+        <v>33.9</v>
+      </c>
+      <c r="N16" s="4" t="inlineStr"/>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>Verified (UiA Coder EPYC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Datacenter Server CPU</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>AMD EPYC 9374F 32-Core Processor</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>x86_64 (Zen 4, 32C/64T)</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Stock YOLOv11s Baseline</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>FP32</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>95.75</v>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>95.75</v>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J17" s="7" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="K17" s="7" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="L17" s="7" t="n">
+        <v>59.76</v>
+      </c>
+      <c r="M17" s="7" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="N17" s="7" t="inlineStr"/>
+      <c r="O17" s="5" t="inlineStr">
+        <is>
+          <t>Verified (UiA Coder EPYC)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: Record physical Rock Pi 4C+ benchmark results across all 7 models
</commit_message>
<xml_diff>
--- a/results/edge_benchmark_results.xlsx
+++ b/results/edge_benchmark_results.xlsx
@@ -470,12 +470,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="37" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
@@ -487,7 +487,7 @@
     <col width="26" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="32" customWidth="1" min="15" max="15"/>
+    <col width="35" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1485,6 +1485,363 @@
         </is>
       </c>
     </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Embedded SBC (ARM)</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Rock Pi 4C+</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Rockchip RK3399 (2x A72 + 4x A53)</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Ours (Hybrid Dilated ECA v30)</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>FP32</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>1314.61</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>1314.61</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I18" s="4" t="inlineStr"/>
+      <c r="J18" s="4" t="inlineStr"/>
+      <c r="K18" s="4" t="inlineStr"/>
+      <c r="L18" s="4" t="n">
+        <v>1238.64</v>
+      </c>
+      <c r="M18" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="N18" s="4" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>Verified (Physical Rock Pi 4C+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Embedded SBC (ARM)</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Rock Pi 4C+</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Rockchip RK3399 (2x A72 + 4x A53)</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Stock YOLOv8n Baseline</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>FP32</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="n">
+        <v>1315.78</v>
+      </c>
+      <c r="G19" s="7" t="n">
+        <v>1315.78</v>
+      </c>
+      <c r="H19" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I19" s="7" t="inlineStr"/>
+      <c r="J19" s="7" t="inlineStr"/>
+      <c r="K19" s="7" t="inlineStr"/>
+      <c r="L19" s="7" t="n">
+        <v>1294.22</v>
+      </c>
+      <c r="M19" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="N19" s="7" t="inlineStr"/>
+      <c r="O19" s="5" t="inlineStr">
+        <is>
+          <t>Verified (Physical Rock Pi 4C+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Embedded SBC (ARM)</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Rock Pi 4C+</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Rockchip RK3399 (2x A72 + 4x A53)</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Stock YOLOv8s Baseline</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>FP32</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>3211.85</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>3211.85</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="inlineStr"/>
+      <c r="L20" s="4" t="n">
+        <v>3176.49</v>
+      </c>
+      <c r="M20" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="N20" s="4" t="inlineStr"/>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>Verified (Physical Rock Pi 4C+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Embedded SBC (ARM)</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Rock Pi 4C+</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Rockchip RK3399 (2x A72 + 4x A53)</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Stock YOLOv10n Baseline</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>FP32</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="n">
+        <v>1708.62</v>
+      </c>
+      <c r="G21" s="7" t="n">
+        <v>1708.62</v>
+      </c>
+      <c r="H21" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I21" s="7" t="inlineStr"/>
+      <c r="J21" s="7" t="inlineStr"/>
+      <c r="K21" s="7" t="inlineStr"/>
+      <c r="L21" s="7" t="n">
+        <v>1596.19</v>
+      </c>
+      <c r="M21" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="N21" s="7" t="inlineStr"/>
+      <c r="O21" s="5" t="inlineStr">
+        <is>
+          <t>Verified (Physical Rock Pi 4C+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Embedded SBC (ARM)</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Rock Pi 4C+</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Rockchip RK3399 (2x A72 + 4x A53)</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Stock YOLOv10s Baseline</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>FP32</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>3814.65</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>3814.65</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I22" s="4" t="inlineStr"/>
+      <c r="J22" s="4" t="inlineStr"/>
+      <c r="K22" s="4" t="inlineStr"/>
+      <c r="L22" s="4" t="n">
+        <v>3173</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="N22" s="4" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>Verified (Physical Rock Pi 4C+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Embedded SBC (ARM)</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Rock Pi 4C+</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Rockchip RK3399 (2x A72 + 4x A53)</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Stock YOLOv11n Baseline</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>FP32</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="n">
+        <v>3136.93</v>
+      </c>
+      <c r="G23" s="7" t="n">
+        <v>3136.93</v>
+      </c>
+      <c r="H23" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I23" s="7" t="inlineStr"/>
+      <c r="J23" s="7" t="inlineStr"/>
+      <c r="K23" s="7" t="inlineStr"/>
+      <c r="L23" s="7" t="n">
+        <v>2852.14</v>
+      </c>
+      <c r="M23" s="7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N23" s="7" t="inlineStr"/>
+      <c r="O23" s="5" t="inlineStr">
+        <is>
+          <t>Verified (Physical Rock Pi 4C+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Embedded SBC (ARM)</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Rock Pi 4C+</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Rockchip RK3399 (2x A72 + 4x A53)</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Stock YOLOv11s Baseline</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>FP32</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>3159.39</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>3159.39</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I24" s="4" t="inlineStr"/>
+      <c r="J24" s="4" t="inlineStr"/>
+      <c r="K24" s="4" t="inlineStr"/>
+      <c r="L24" s="4" t="n">
+        <v>3150.24</v>
+      </c>
+      <c r="M24" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="N24" s="4" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>Verified (Physical Rock Pi 4C+)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: Record physical Raspberry Pi 4B benchmark results
</commit_message>
<xml_diff>
--- a/results/edge_benchmark_results.xlsx
+++ b/results/edge_benchmark_results.xlsx
@@ -470,10 +470,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="37" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" min="4" max="4"/>
@@ -487,7 +487,7 @@
     <col width="26" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="35" customWidth="1" min="15" max="15"/>
+    <col width="52" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1842,6 +1842,200 @@
         </is>
       </c>
     </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Low-Power Edge SBC (ARM)</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Raspberry Pi 4B</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Broadcom BCM2711 (4x Cortex-A72)</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Ours (Hybrid Dilated ECA v30)</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>FP32</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="n">
+        <v>1179.16</v>
+      </c>
+      <c r="G25" s="7" t="n">
+        <v>1179.16</v>
+      </c>
+      <c r="H25" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I25" s="7" t="inlineStr"/>
+      <c r="J25" s="7" t="inlineStr"/>
+      <c r="K25" s="7" t="inlineStr"/>
+      <c r="L25" s="7" t="n">
+        <v>970.76</v>
+      </c>
+      <c r="M25" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N25" s="7" t="inlineStr"/>
+      <c r="O25" s="5" t="inlineStr">
+        <is>
+          <t>Verified (Physical Raspberry Pi 4B)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Low-Power Edge SBC (ARM)</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Raspberry Pi 4B</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Broadcom BCM2711 (4x Cortex-A72)</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Stock YOLOv8n Baseline</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>FP32</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>963.26</v>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>963.26</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" s="4" t="inlineStr"/>
+      <c r="J26" s="4" t="inlineStr"/>
+      <c r="K26" s="4" t="inlineStr"/>
+      <c r="L26" s="4" t="n">
+        <v>991.13</v>
+      </c>
+      <c r="M26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N26" s="4" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>Verified (Physical Raspberry Pi 4B)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Low-Power Edge SBC (ARM)</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Raspberry Pi 4B</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Broadcom BCM2711 (4x Cortex-A72)</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Stock YOLOv8s Baseline</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>FP32</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="n">
+        <v>2382.64</v>
+      </c>
+      <c r="G27" s="7" t="n">
+        <v>2382.64</v>
+      </c>
+      <c r="H27" s="7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I27" s="7" t="inlineStr"/>
+      <c r="J27" s="7" t="inlineStr"/>
+      <c r="K27" s="7" t="inlineStr"/>
+      <c r="L27" s="7" t="n">
+        <v>2361.25</v>
+      </c>
+      <c r="M27" s="7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N27" s="7" t="inlineStr"/>
+      <c r="O27" s="5" t="inlineStr">
+        <is>
+          <t>Verified (Physical Raspberry Pi 4B)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Low-Power Edge SBC (ARM)</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Raspberry Pi 4B</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Broadcom BCM2711 (4x Cortex-A72)</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Stock YOLOv10n Baseline</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>FP32</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr"/>
+      <c r="G28" s="4" t="inlineStr"/>
+      <c r="H28" s="4" t="inlineStr"/>
+      <c r="I28" s="4" t="inlineStr"/>
+      <c r="J28" s="4" t="inlineStr"/>
+      <c r="K28" s="4" t="inlineStr"/>
+      <c r="L28" s="4" t="inlineStr"/>
+      <c r="M28" s="4" t="inlineStr"/>
+      <c r="N28" s="4" t="inlineStr"/>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>Incompatible (Illegal Instruction on Cortex-A72)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>